<commit_message>
Added the calculator to unit converter
</commit_message>
<xml_diff>
--- a/RoadMap/AI Engineer Tracking Sheet.xlsx
+++ b/RoadMap/AI Engineer Tracking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e889d5051bb0329/ドキュメント/AIML/RoadMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_0FB22D5A0AE9A8480E28AC64B768C8CE979C262B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A9CEB39-7487-473E-A460-47C5B8680256}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_0FB22D5A0AE9A8480E28AC64B768C8CE979C262B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AF936F4-ADC7-446F-9CA1-B4F02FE4A973}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="855" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="B3" s="2">
         <f>COUNTIF('Daily Tracker'!I:I,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B4" s="6">
         <f>B3/B2</f>
-        <v>1.1111111111111112E-2</v>
+        <v>1.6666666666666666E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
@@ -3109,7 +3109,7 @@
         <v>65</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>66</v>
+        <v>501</v>
       </c>
       <c r="J4" s="5">
         <v>2.5</v>

</xml_diff>

<commit_message>
completed upto day 7
</commit_message>
<xml_diff>
--- a/RoadMap/AI Engineer Tracking Sheet.xlsx
+++ b/RoadMap/AI Engineer Tracking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e889d5051bb0329/ドキュメント/AIML/RoadMap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_0FB22D5A0AE9A8480E28AC64B768C8CE979C262B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7525A842-6B29-47D7-96BC-7E696F49B316}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_0FB22D5A0AE9A8480E28AC64B768C8CE979C262B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB239CCF-3DE0-4E8C-A254-563BACA99F1A}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="855" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="B3" s="2">
         <f>COUNTIF('Daily Tracker'!I:I,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B4" s="6">
         <f>B3/B2</f>
-        <v>2.2222222222222223E-2</v>
+        <v>2.7777777777777776E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
@@ -3175,7 +3175,7 @@
         <v>65</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>66</v>
+        <v>501</v>
       </c>
       <c r="J6" s="5">
         <v>2.5</v>

</xml_diff>